<commit_message>
Remove duplicate late-evening loading message
"Winding down after a long day in the field." was dropped from the
9pm-midnight loading pool; syncs the spreadsheet source of truth with the
already-edited catalog JSON.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>Winding down after a long day in the field.</t>
+          <t>Night falls over the hive.</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>Night falls over the hive.</t>
+          <t>The comb quietens as the stars come out.</t>
         </is>
       </c>
       <c r="D24" s="1" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>The comb quietens as the stars come out.</t>
+          <t>Just one more game... famous last words in the hive.</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
@@ -1909,12 +1909,12 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 9:00 PM and midnight local time.</t>
+          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>Just one more game... famous last words in the hive.</t>
+          <t>Morning in the comb — the day's first harvest begins!</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>Morning in the comb — the day's first harvest begins!</t>
+          <t>Peak pollen-gathering hours!</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Peak pollen-gathering hours!</t>
+          <t>The hive is buzzing with morning energy.</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
+          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>The hive is buzzing with morning energy.</t>
+          <t>High noon in the hive — time for a honey break!</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>High noon in the hive — time for a honey break!</t>
+          <t>The sun is high, and the nectar is sweet.</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>The sun is high, and the nectar is sweet.</t>
+          <t>Midday match! A quick break between flights.</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
@@ -2071,12 +2071,12 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
+          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>Midday match! A quick break between flights.</t>
+          <t>Golden afternoon light fills the comb.</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>Golden afternoon light fills the comb.</t>
+          <t>The afternoon warmth has the bees buzzing lively.</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>The afternoon warmth has the bees buzzing lively.</t>
+          <t>Basking in the warm afternoon sun.</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>Basking in the warm afternoon sun.</t>
+          <t>The sun sets over the hive — time for evening games.</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>The sun sets over the hive — time for evening games.</t>
+          <t>Workers return home after a full day's buzz.</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>Workers return home after a full day's buzz.</t>
+          <t>Golden hour in the honeycomb.</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
@@ -2226,27 +2226,27 @@
       </c>
     </row>
     <row r="38" ht="14.6" customHeight="1" s="8">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B38" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C38" s="1" t="inlineStr">
-        <is>
-          <t>Golden hour in the honeycomb.</t>
-        </is>
-      </c>
-      <c r="D38" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E38" s="1" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>On Game Load</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Warming up flights muscles…</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Warming up flights muscles…</t>
+          <t>Pollinating the processors…</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Pollinating the processors…</t>
+          <t>Untangling waggle-dance choreography…</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Untangling waggle-dance choreography…</t>
+          <t>Generating royal jelly…</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Generating royal jelly…</t>
+          <t>Sealing the honeycomb…</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Sealing the honeycomb…</t>
+          <t>Consulting the Queen Bee…</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Consulting the Queen Bee…</t>
+          <t>Calibrating stingers…</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Calibrating stingers…</t>
+          <t>Deploying scout bees…</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Deploying scout bees…</t>
+          <t>Counting the worker bees…</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Counting the worker bees…</t>
+          <t>Preparing a sticky situation…</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Preparing a sticky situation…</t>
+          <t>The swarm is gathering…</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>The swarm is gathering…</t>
+          <t>Sweeping the hive…</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Sweeping the hive…</t>
+          <t>Gathering nectar from local memory…</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Gathering nectar from local memory…</t>
+          <t>Guarding the entrance from wasps…</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Guarding the entrance from wasps…</t>
+          <t>Feeding the larvae bits and bytes…</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Feeding the larvae bits and bytes…</t>
+          <t>Orienting new forager bees…</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Orienting new forager bees…</t>
+          <t>Cross-referencing pollen routes…</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Cross-referencing pollen routes…</t>
+          <t>Recruiting nurse bees…</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Recruiting nurse bees…</t>
+          <t>Loading nectar reserves…</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Loading nectar reserves…</t>
+          <t>Synchronizing with the hive mind…</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Synchronizing with the hive mind…</t>
+          <t>Tuning antennae for reception…</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Tuning antennae for reception…</t>
+          <t>Propolis-sealing the cracks…</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Propolis-sealing the cracks…</t>
+          <t>Rousing drones from their nap…</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2849,27 +2849,27 @@
     <row r="61" ht="14.6" customHeight="1" s="8">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>On Game Load</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Rousing drones from their nap…</t>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>The hive hums quietly, waiting for your next move.</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>Loading</t>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Toast</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>The hive hums quietly, waiting for your next move.</t>
+          <t>A stray bee drifts across the board...</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>A stray bee drifts across the board...</t>
+          <t>It’s when you can’t hear the bees, that’s when the bees are coming.</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>It’s when you can’t hear the bees, that’s when the bees are coming.</t>
+          <t>Somewhere, honey is dripping.</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Somewhere, honey is dripping.</t>
+          <t>The comb creaks softly under the weight of gathered honey.</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>The comb creaks softly under the weight of gathered honey.</t>
+          <t>A distant hum grows louder... or is that just the board?</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>A distant hum grows louder... or is that just the board?</t>
+          <t>Pollen settles on the board like fine snow.</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -3046,12 +3046,12 @@
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Pollen settles on the board like fine snow.</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Somewhere, a queen bee hums a low, satisfied note.</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Somewhere, a queen bee hums a low, satisfied note.</t>
+          <t>The board glows faintly gold in the afternoon light.</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>The board glows faintly gold in the afternoon light.</t>
+          <t>A single petal drifts down onto the comb.</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>A single petal drifts down onto the comb.</t>
+          <t>The hive never truly sleeps.</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -3154,12 +3154,12 @@
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>The hive never truly sleeps.</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>The swarm is silently judging your strategy.</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
@@ -3181,9 +3181,9 @@
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>The swarm is silently judging your strategy.</t>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>A worker bee pauses mid-flight, unsure why.</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>A worker bee pauses mid-flight, unsure why.</t>
+          <t>Somewhere, a bee is telling the others where you’ve been.</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Somewhere, a bee is telling the others where you’ve been.</t>
+          <t>The hive remembers every card you’ve touched.</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>The hive remembers every card you’ve touched.</t>
+          <t>Nothing moves. Everything hums.</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Nothing moves. Everything hums.</t>
+          <t>The edges of the cards are getting a little sticky.</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>The edges of the cards are getting a little sticky.</t>
+          <t>The bees are keeping score. They always do.</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>The bees are keeping score. They always do.</t>
+          <t>A bee lands, looks around, and leaves again.</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>A bee lands, looks around, and leaves again.</t>
+          <t>The hum has changed pitch. Did you notice?</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>The hum has changed pitch. Did you notice?</t>
+          <t>Time moves differently inside the comb.</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Time moves differently inside the comb.</t>
+          <t>Somewhere, wax is being warmed by tiny bodies.</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Somewhere, wax is being warmed by tiny bodies.</t>
+          <t>Even idle hands make honey eventually.</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Even idle hands make honey eventually.</t>
+          <t>The bees are patient. Are you?</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>The bees are patient. Are you?</t>
+          <t>The hive keeps its own time.</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3524,52 +3524,52 @@
     <row r="86" ht="14.6" customHeight="1" s="8">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Idle Action</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>No action taken for one minute.</t>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>3+ Hints used in one match.</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>The hive keeps its own time.</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>Ambiance</t>
-        </is>
-      </c>
-      <c r="E86" s="4" t="inlineStr">
+          <t>Need a little help? The scout bees are buzzing suggestions.</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="87" ht="14.6" customHeight="1" s="8">
-      <c r="A87" s="5" t="inlineStr">
+      <c r="A87" s="1" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B87" s="5" t="inlineStr">
+      <c r="B87" s="1" t="inlineStr">
         <is>
           <t>3+ Hints used in one match.</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Need a little help? The scout bees are buzzing suggestions.</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="inlineStr">
+      <c r="C87" s="1" t="inlineStr">
+        <is>
+          <t>Waggle dance activated!</t>
+        </is>
+      </c>
+      <c r="D87" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E87" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>Waggle dance activated!</t>
+          <t>The bees checked every flower!</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>The bees checked every flower!</t>
+          <t>The hive mind is thinking...</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>The hive mind is thinking...</t>
+          <t>The hive has reached a consensus.</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>The hive has reached a consensus.</t>
+          <t>Even the busiest bees ask the Queen for directions sometimes.</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>Even the busiest bees ask the Queen for directions sometimes.</t>
+          <t>A drop of honey marks a sweet path forward.</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>A drop of honey marks a sweet path forward.</t>
+          <t>Nectar trail spotted! Follow this lead.</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>Nectar trail spotted! Follow this lead.</t>
+          <t>A little bee whispered a suggestion in your ear.</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
@@ -3765,54 +3765,54 @@
       </c>
     </row>
     <row r="95" ht="14.6" customHeight="1" s="8">
-      <c r="A95" s="1" t="inlineStr">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B95" s="1" t="inlineStr">
-        <is>
-          <t>3+ Hints used in one match.</t>
-        </is>
-      </c>
-      <c r="C95" s="1" t="inlineStr">
-        <is>
-          <t>A little bee whispered a suggestion in your ear.</t>
-        </is>
-      </c>
-      <c r="D95" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E95" s="1" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Undo used immediately after a placement.</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Second thoughts? Wise bees always double-check.</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="96" ht="14.6" customHeight="1" s="8">
-      <c r="A96" s="5" t="inlineStr">
+      <c r="A96" s="1" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B96" s="5" t="inlineStr">
+      <c r="B96" s="1" t="inlineStr">
         <is>
           <t>Undo used immediately after a placement.</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>Second thoughts? Wise bees always double-check.</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
+      <c r="C96" s="1" t="inlineStr">
+        <is>
+          <t>Re-charting the swarm!</t>
+        </is>
+      </c>
+      <c r="D96" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E96" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>Re-charting the swarm!</t>
+          <t>Mid-air flight recalculation!</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>Mid-air flight recalculation!</t>
+          <t>Hovering backwards...</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>Hovering backwards...</t>
+          <t>Plucking that card right back out of the wax.</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>Plucking that card right back out of the wax.</t>
+          <t>Unsticking that card from the comb.</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
@@ -3927,46 +3927,46 @@
       </c>
     </row>
     <row r="101" ht="14.6" customHeight="1" s="8">
-      <c r="A101" s="1" t="inlineStr">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B101" s="1" t="inlineStr">
-        <is>
-          <t>Undo used immediately after a placement.</t>
-        </is>
-      </c>
-      <c r="C101" s="1" t="inlineStr">
-        <is>
-          <t>Unsticking that card from the comb.</t>
-        </is>
-      </c>
-      <c r="D101" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E101" s="1" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Player wins a match with 4 rules active at once.</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Four rules, one victory. Chaos bends to you.</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="102" ht="14.6" customHeight="1" s="8">
-      <c r="A102" s="5" t="inlineStr">
+      <c r="A102" s="3" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>Player wins a match with 4 rules active at once.</t>
-        </is>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>Four rules, one victory. Chaos bends to you.</t>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Opponent is winning by two cards and is about to place the last card on the board.</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>{OpponentName} prepares a final sting!</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -3988,12 +3988,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Opponent is winning by two cards and is about to place the last card on the board.</t>
+          <t>Player flips 3+ cards in a single turn.</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>{OpponentName} prepares a final sting!</t>
+          <t>A massive swarm!</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -4015,12 +4015,12 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Player flips 3+ cards in a single turn.</t>
+          <t>Opponent flips 3+ of the player's cards in a single turn (not a Combo).</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>A massive swarm!</t>
+          <t>{OpponentName} unleashes an angry swarm!</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Opponent flips 3+ of the player's cards in a single turn (not a Combo).</t>
+          <t>Combo x4 or higher.</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>{OpponentName} unleashes an angry swarm!</t>
+          <t>SWARM FRENZY — the whole hive is buzzing!</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -4069,12 +4069,12 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Combo x4 or higher.</t>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>SWARM FRENZY — the whole hive is buzzing!</t>
+          <t>The hive is nearly overrun... is there any hope left?</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -4096,12 +4096,12 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+          <t>A placed card captures on all 4 sides at once.</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>The hive is nearly overrun... is there any hope left?</t>
+          <t>Four-way sting!</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -4116,22 +4116,22 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="3" t="inlineStr">
+      <c r="A108" s="5" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>A placed card captures on all 4 sides at once.</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>Four-way sting!</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>{OpponentName} is starting to sweat.</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
         <is>
           <t>Repeatable Flavor</t>
         </is>
@@ -4150,12 +4150,12 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>3+ rematch wins in a row against the same opponent.</t>
+          <t>3+ rematch losses in a row against the same opponent.</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>{OpponentName} is starting to sweat.</t>
+          <t>{OpponentName} has your number. Time for a new strategy?</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
@@ -4177,12 +4177,12 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>3+ rematch losses in a row against the same opponent.</t>
+          <t>A 1-star card captures 3+ cards in one move.</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>{OpponentName} has your number. Time for a new strategy?</t>
+          <t>The weakest bee just took down half the hive!</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -4204,12 +4204,12 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>A 1-star card captures 3+ cards in one move.</t>
+          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>The weakest bee just took down half the hive!</t>
+          <t>A worker bee just humbled royalty.</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -4224,22 +4224,22 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="inlineStr">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>A worker bee just humbled royalty.</t>
-        </is>
-      </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Second thoughts... wait, never mind, let's stick to the plan.</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
         <is>
           <t>Repeatable Flavor</t>
         </is>
@@ -4258,12 +4258,12 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+          <t>Player plays against the same AI difficulty 5 times in a row.</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Second thoughts... wait, never mind, let's stick to the plan.</t>
+          <t>A true rivalry is forming in the comb.</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -4285,12 +4285,12 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Player plays against the same AI difficulty 5 times in a row.</t>
+          <t>Player wins by the maximum possible margin.</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>A true rivalry is forming in the comb.</t>
+          <t>Nothing left to sting!</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -4307,25 +4307,25 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>Player wins by the maximum possible margin.</t>
-        </is>
-      </c>
-      <c r="C115" s="3" t="inlineStr">
-        <is>
-          <t>Nothing left to sting!</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E115" s="6" t="inlineStr">
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>First launch ever</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>A new bee joins the hive. Thank you for playing!</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>Achievement</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4339,12 +4339,12 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>First launch ever</t>
+          <t>Player reaches 10 total wins.</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>A new bee joins the hive. Thank you for playing!</t>
+          <t>10 wins. The hive takes notice.</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
@@ -4366,12 +4366,12 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>Player reaches 10 total wins.</t>
+          <t>Player reaches 100 total wins.</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>10 wins. The hive takes notice.</t>
+          <t>100 wins. The colony sings your name.</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -4393,12 +4393,12 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>Player reaches 100 total wins.</t>
+          <t>Player reaches 1000 total wins.</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>100 wins. The colony sings your name.</t>
+          <t>1000 wins. The hive bends to your will.</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -4415,22 +4415,22 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>Player reaches 1000 total wins.</t>
-        </is>
-      </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>1000 wins. The hive bends to your will.</t>
-        </is>
-      </c>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t>Achievement</t>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Fallen Ace triggers (a '1' captures a '10').</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>The drone takes down the Queen!</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>The drone takes down the Queen!</t>
+          <t>A lucky sting! The mighty have fallen.</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -4467,27 +4467,27 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="3" t="inlineStr">
+      <c r="A121" s="5" t="inlineStr">
         <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>Fallen Ace triggers (a '1' captures a '10').</t>
-        </is>
-      </c>
-      <c r="C121" s="3" t="inlineStr">
-        <is>
-          <t>A lucky sting! The mighty have fallen.</t>
-        </is>
-      </c>
-      <c r="D121" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Pollination pushes a card's modifier to +3 or higher.</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>The pollen's thick today — {AscensionSuit} is in full bloom!</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4501,12 +4501,12 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Pollination pushes a card's modifier to +3 or higher.</t>
+          <t>Smoked Out drops a card's effective stat to 1.</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>The pollen's thick today — {AscensionSuit} is in full bloom!</t>
+          <t>Smoked out — that card can barely buzz anymore.</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -4521,56 +4521,56 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="inlineStr">
+      <c r="A123" s="3" t="inlineStr">
         <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>Smoked Out drops a card's effective stat to 1.</t>
-        </is>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>Smoked out — that card can barely buzz anymore.</t>
-        </is>
-      </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E123" s="6" t="inlineStr">
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>A player triggers a "Plus" combo (the math matches perfectly).</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>The math checks out!</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="3" t="inlineStr">
+      <c r="A124" s="5" t="inlineStr">
         <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
-        <is>
-          <t>A player triggers a "Plus" combo (the math matches perfectly).</t>
-        </is>
-      </c>
-      <c r="C124" s="3" t="inlineStr">
-        <is>
-          <t>The math checks out!</t>
-        </is>
-      </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr">
-        <is>
-          <t>Toast</t>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Player wins flawless (opponent score = 0).</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Flawless victory!</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>Win Banner</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Flawless victory!</t>
+          <t>Hive domination!</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>Hive domination!</t>
+          <t>The colony reigns supreme..</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
@@ -4636,12 +4636,12 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Player wins flawless (opponent score = 0).</t>
+          <t>Player loses flawless (0 captures).</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>The colony reigns supreme..</t>
+          <t>Every card fell. The hive lies in ruins.</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>Win Banner</t>
+          <t>You Lose Banner</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>Every card fell. The hive lies in ruins.</t>
+          <t>{OpponentName} didn't leave you a single card standing.</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>{OpponentName} didn't leave you a single card standing.</t>
+          <t>There are no bees left in your bonnet.</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
@@ -4715,14 +4715,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>Player loses flawless (0 captures).</t>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Roulette rolls Pollination.</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>There are no bees left in your bonnet.</t>
+          <t>Pollen is in the air!</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="E130" s="6" t="inlineStr">
         <is>
-          <t>You Lose Banner</t>
+          <t>Game intro rules banner</t>
         </is>
       </c>
     </row>
@@ -4744,12 +4744,12 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Roulette rolls Pollination.</t>
+          <t>Roulette rolls Smoked Out.</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Pollen is in the air!</t>
+          <t>A haze covers the comb!</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -4769,14 +4769,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B132" s="3" t="inlineStr">
-        <is>
-          <t>Roulette rolls Smoked Out.</t>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Roulette rolls Math Bee</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>A haze covers the comb!</t>
+          <t>Addition is key!</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
@@ -4798,12 +4798,12 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Math Bee</t>
+          <t>Roulette rolls Inversion</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Addition is key!</t>
+          <t>Everything is upside down!</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
@@ -4825,12 +4825,12 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Inversion</t>
+          <t>Roulette rolls clear skies</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Everything is upside down!</t>
+          <t>The hive is exposed!</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
@@ -4852,12 +4852,12 @@
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls clear skies</t>
+          <t>Roulette rolls scouting party</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>The hive is exposed!</t>
+          <t>The drones are out!</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
@@ -4879,12 +4879,12 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls scouting party</t>
+          <t>Roulette rolls Frenzy</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>The drones are out!</t>
+          <t>Chaos takes over!</t>
         </is>
       </c>
       <c r="D136" s="6" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Frenzy</t>
+          <t>Roulette rolls Symmetry</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Chaos takes over!</t>
+          <t>Patterns Align!</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
@@ -4933,12 +4933,12 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Symmetry</t>
+          <t>Roulette rolls Nectar Exchange</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>Patterns Align!</t>
+          <t>A trade before the swarm!</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
@@ -4960,12 +4960,12 @@
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Nectar Exchange</t>
+          <t>Roulette rolls Hierarchy</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>A trade before the swarm!</t>
+          <t>Order above all!</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
@@ -4980,324 +4980,297 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="5" t="inlineStr">
-        <is>
-          <t>Rule-Specific</t>
-        </is>
-      </c>
-      <c r="B140" s="5" t="inlineStr">
-        <is>
-          <t>Roulette rolls Hierarchy</t>
-        </is>
-      </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>Order above all!</t>
-        </is>
-      </c>
-      <c r="D140" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E140" s="6" t="inlineStr">
-        <is>
-          <t>Game intro rules banner</t>
+      <c r="A140" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B140" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+        </is>
+      </c>
+      <c r="C140" s="1" t="inlineStr">
+        <is>
+          <t>Moonlight glints off the wax.</t>
+        </is>
+      </c>
+      <c r="D140" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E140" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Moonlight glints off the wax.</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 5:00 AM and 8:00 AM local time.</t>
+        </is>
+      </c>
+      <c r="C141" s="1" t="inlineStr">
+        <is>
+          <t>The dew hasn't dried and the bees are already at it.</t>
+        </is>
+      </c>
+      <c r="D141" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E141" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Match starts between 5:00 AM and 8:00 AM local time.</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>The dew hasn't dried and the bees are already at it.</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
+      <c r="A142" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B142" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C142" s="1" t="inlineStr">
+        <is>
+          <t>The hive hums with a fresh day's plans.</t>
+        </is>
+      </c>
+      <c r="D142" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E142" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>The hive hums with a fresh day's plans.</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
+      <c r="A143" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B143" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C143" s="1" t="inlineStr">
+        <is>
+          <t>Even bees pause to enjoy the sunshine.</t>
+        </is>
+      </c>
+      <c r="D143" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E143" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B144" s="1" t="inlineStr">
         <is>
           <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Even bees pause to enjoy the sunshine.</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
+      <c r="C144" s="1" t="inlineStr">
+        <is>
+          <t>Half the day's pollen is already in.</t>
+        </is>
+      </c>
+      <c r="D144" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E144" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Half the day's pollen is already in.</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B145" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C145" s="1" t="inlineStr">
+        <is>
+          <t>The hive settles into its afternoon rhythm.</t>
+        </is>
+      </c>
+      <c r="D145" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E145" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
+      <c r="A146" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B146" s="1" t="inlineStr">
         <is>
           <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>The hive settles into its afternoon rhythm.</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
+      <c r="C146" s="1" t="inlineStr">
+        <is>
+          <t>Long shadows, long odds — let's play.</t>
+        </is>
+      </c>
+      <c r="D146" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E146" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Long shadows, long odds — let's play.</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C147" s="1" t="inlineStr">
+        <is>
+          <t>The last foragers are heading home.</t>
+        </is>
+      </c>
+      <c r="D147" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E147" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="inlineStr">
         <is>
           <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>The last foragers are heading home.</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
+      <c r="C148" s="1" t="inlineStr">
+        <is>
+          <t>Lantern-bugs light the way to the hive.</t>
+        </is>
+      </c>
+      <c r="D148" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E148" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Lantern-bugs light the way to the hive.</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 9:00 PM and midnight local time.</t>
+        </is>
+      </c>
+      <c r="C149" s="1" t="inlineStr">
+        <is>
+          <t>The Queen's chambers go quiet, but not this table.</t>
+        </is>
+      </c>
+      <c r="D149" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E149" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B150" s="1" t="inlineStr">
         <is>
           <t>Match starts between 9:00 PM and midnight local time.</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>The Queen's chambers go quiet, but not this table.</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Match starts between 9:00 PM and midnight local time.</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
+      <c r="C150" s="1" t="inlineStr">
         <is>
           <t>A nightcap of nectar before bed.</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
+      <c r="D150" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E150" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>

</xml_diff>

<commit_message>
Add 5 more variants to the undo-repeat-move banner
Player uses Undo, thinks about it, and then makes the exact same move
they just undid — was a single-message trigger, now has 6 variants to
cycle through. Edited the spreadsheet and regenerated both platforms'
catalog JSON via tools/generate_banner_catalog.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -4251,135 +4251,135 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>Player plays against the same AI difficulty 5 times in a row.</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>A true rivalry is forming in the comb.</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E113" s="6" t="inlineStr">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>A worker bee never doubts their instincts... twice!</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="3" t="inlineStr">
+      <c r="A114" t="inlineStr">
         <is>
           <t>Gameplay</t>
         </is>
       </c>
-      <c r="B114" s="3" t="inlineStr">
-        <is>
-          <t>Player wins by the maximum possible margin.</t>
-        </is>
-      </c>
-      <c r="C114" s="3" t="inlineStr">
-        <is>
-          <t>Nothing left to sting!</t>
-        </is>
-      </c>
-      <c r="D114" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Just testing the Undo button, right?</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>First launch ever</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>A new bee joins the hive. Thank you for playing!</t>
-        </is>
-      </c>
-      <c r="D115" s="7" t="inlineStr">
-        <is>
-          <t>Achievement</t>
-        </is>
-      </c>
-      <c r="E115" s="7" t="inlineStr">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>You just wanted to see that card flip again!</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="3" t="inlineStr">
-        <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>Player reaches 10 total wins.</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>10 wins. The hive takes notice.</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t>Achievement</t>
-        </is>
-      </c>
-      <c r="E116" s="7" t="inlineStr">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>A plot twist... that went absolutely nowhere!</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="3" t="inlineStr">
-        <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Player reaches 100 total wins.</t>
-        </is>
-      </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>100 wins. The colony sings your name.</t>
-        </is>
-      </c>
-      <c r="D117" s="7" t="inlineStr">
-        <is>
-          <t>Achievement</t>
-        </is>
-      </c>
-      <c r="E117" s="7" t="inlineStr">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Taking the scenic route to the exact same move!</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4388,25 +4388,25 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>Player reaches 1000 total wins.</t>
-        </is>
-      </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>1000 wins. The hive bends to your will.</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t>Achievement</t>
-        </is>
-      </c>
-      <c r="E118" s="7" t="inlineStr">
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Player plays against the same AI difficulty 5 times in a row.</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>A true rivalry is forming in the comb.</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E118" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4415,17 +4415,17 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Rule-Specific</t>
+          <t>Gameplay</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Fallen Ace triggers (a '1' captures a '10').</t>
+          <t>Player wins by the maximum possible margin.</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>The drone takes down the Queen!</t>
+          <t>Nothing left to sting!</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -4433,7 +4433,7 @@
           <t>Repeatable Flavor</t>
         </is>
       </c>
-      <c r="E119" s="7" t="inlineStr">
+      <c r="E119" s="6" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4442,22 +4442,22 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Rule-Specific</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="inlineStr">
-        <is>
-          <t>Fallen Ace triggers (a '1' captures a '10').</t>
-        </is>
-      </c>
-      <c r="C120" s="3" t="inlineStr">
-        <is>
-          <t>A lucky sting! The mighty have fallen.</t>
-        </is>
-      </c>
-      <c r="D120" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>First launch ever</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>A new bee joins the hive. Thank you for playing!</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>Achievement</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
@@ -4467,54 +4467,54 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr">
-        <is>
-          <t>Rule-Specific</t>
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Milestones</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Pollination pushes a card's modifier to +3 or higher.</t>
+          <t>Player reaches 10 total wins.</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>The pollen's thick today — {AscensionSuit} is in full bloom!</t>
-        </is>
-      </c>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E121" s="6" t="inlineStr">
+          <t>10 wins. The hive takes notice.</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Achievement</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>Rule-Specific</t>
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>Milestones</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Smoked Out drops a card's effective stat to 1.</t>
+          <t>Player reaches 100 total wins.</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Smoked out — that card can barely buzz anymore.</t>
-        </is>
-      </c>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E122" s="6" t="inlineStr">
+          <t>100 wins. The colony sings your name.</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>Achievement</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -4523,81 +4523,81 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Player reaches 1000 total wins.</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>1000 wins. The hive bends to your will.</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t>Achievement</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>A player triggers a "Plus" combo (the math matches perfectly).</t>
-        </is>
-      </c>
-      <c r="C123" s="3" t="inlineStr">
-        <is>
-          <t>The math checks out!</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E123" s="4" t="inlineStr">
-        <is>
-          <t>Toast</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="5" t="inlineStr">
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Fallen Ace triggers (a '1' captures a '10').</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>The drone takes down the Queen!</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
         <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>Player wins flawless (opponent score = 0).</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>Flawless victory!</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E124" s="6" t="inlineStr">
-        <is>
-          <t>Win Banner</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t>Rule-Specific</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
-        <is>
-          <t>Player wins flawless (opponent score = 0).</t>
-        </is>
-      </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>Hive domination!</t>
-        </is>
-      </c>
-      <c r="D125" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E125" s="6" t="inlineStr">
-        <is>
-          <t>Win Banner</t>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Fallen Ace triggers (a '1' captures a '10').</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>A lucky sting! The mighty have fallen.</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="inlineStr">
+        <is>
+          <t>Toast</t>
         </is>
       </c>
     </row>
@@ -4609,12 +4609,12 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>Player wins flawless (opponent score = 0).</t>
+          <t>Pollination pushes a card's modifier to +3 or higher.</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>The colony reigns supreme..</t>
+          <t>The pollen's thick today — {AscensionSuit} is in full bloom!</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="E126" s="6" t="inlineStr">
         <is>
-          <t>Win Banner</t>
+          <t>Toast</t>
         </is>
       </c>
     </row>
@@ -4636,12 +4636,12 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Player loses flawless (0 captures).</t>
+          <t>Smoked Out drops a card's effective stat to 1.</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Every card fell. The hive lies in ruins.</t>
+          <t>Smoked out — that card can barely buzz anymore.</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
@@ -4651,34 +4651,34 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>You Lose Banner</t>
+          <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="inlineStr">
+      <c r="A128" s="3" t="inlineStr">
         <is>
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B128" s="5" t="inlineStr">
-        <is>
-          <t>Player loses flawless (0 captures).</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>{OpponentName} didn't leave you a single card standing.</t>
-        </is>
-      </c>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E128" s="6" t="inlineStr">
-        <is>
-          <t>You Lose Banner</t>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>A player triggers a "Plus" combo (the math matches perfectly).</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>The math checks out!</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>Toast</t>
         </is>
       </c>
     </row>
@@ -4690,12 +4690,12 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Player loses flawless (0 captures).</t>
+          <t>Player wins flawless (opponent score = 0).</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>There are no bees left in your bonnet.</t>
+          <t>Flawless victory!</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>You Lose Banner</t>
+          <t>Win Banner</t>
         </is>
       </c>
     </row>
@@ -4715,14 +4715,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B130" s="3" t="inlineStr">
-        <is>
-          <t>Roulette rolls Pollination.</t>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Player wins flawless (opponent score = 0).</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>Pollen is in the air!</t>
+          <t>Hive domination!</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="E130" s="6" t="inlineStr">
         <is>
-          <t>Game intro rules banner</t>
+          <t>Win Banner</t>
         </is>
       </c>
     </row>
@@ -4742,14 +4742,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
-        <is>
-          <t>Roulette rolls Smoked Out.</t>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Player wins flawless (opponent score = 0).</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>A haze covers the comb!</t>
+          <t>The colony reigns supreme..</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>Game intro rules banner</t>
+          <t>Win Banner</t>
         </is>
       </c>
     </row>
@@ -4771,12 +4771,12 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Math Bee</t>
+          <t>Player loses flawless (0 captures).</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>Addition is key!</t>
+          <t>Every card fell. The hive lies in ruins.</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>Game intro rules banner</t>
+          <t>You Lose Banner</t>
         </is>
       </c>
     </row>
@@ -4798,12 +4798,12 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Inversion</t>
+          <t>Player loses flawless (0 captures).</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Everything is upside down!</t>
+          <t>{OpponentName} didn't leave you a single card standing.</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>Game intro rules banner</t>
+          <t>You Lose Banner</t>
         </is>
       </c>
     </row>
@@ -4825,12 +4825,12 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls clear skies</t>
+          <t>Player loses flawless (0 captures).</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>The hive is exposed!</t>
+          <t>There are no bees left in your bonnet.</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>Game intro rules banner</t>
+          <t>You Lose Banner</t>
         </is>
       </c>
     </row>
@@ -4850,14 +4850,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B135" s="5" t="inlineStr">
-        <is>
-          <t>Roulette rolls scouting party</t>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Roulette rolls Pollination.</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>The drones are out!</t>
+          <t>Pollen is in the air!</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
@@ -4877,14 +4877,14 @@
           <t>Rule-Specific</t>
         </is>
       </c>
-      <c r="B136" s="5" t="inlineStr">
-        <is>
-          <t>Roulette rolls Frenzy</t>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Roulette rolls Smoked Out.</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>Chaos takes over!</t>
+          <t>A haze covers the comb!</t>
         </is>
       </c>
       <c r="D136" s="6" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Symmetry</t>
+          <t>Roulette rolls Math Bee</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Patterns Align!</t>
+          <t>Addition is key!</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
@@ -4933,12 +4933,12 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Roulette rolls Nectar Exchange</t>
+          <t>Roulette rolls Inversion</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>A trade before the swarm!</t>
+          <t>Everything is upside down!</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
@@ -4960,157 +4960,157 @@
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
+          <t>Roulette rolls clear skies</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>The hive is exposed!</t>
+        </is>
+      </c>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E139" s="6" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Roulette rolls scouting party</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>The drones are out!</t>
+        </is>
+      </c>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E140" s="6" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Roulette rolls Frenzy</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Chaos takes over!</t>
+        </is>
+      </c>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Roulette rolls Symmetry</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Patterns Align!</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E142" s="6" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Roulette rolls Nectar Exchange</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>A trade before the swarm!</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
           <t>Roulette rolls Hierarchy</t>
         </is>
       </c>
-      <c r="C139" s="5" t="inlineStr">
+      <c r="C144" s="5" t="inlineStr">
         <is>
           <t>Order above all!</t>
         </is>
       </c>
-      <c r="D139" s="6" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E139" s="6" t="inlineStr">
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="inlineStr">
         <is>
           <t>Game intro rules banner</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B140" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
-        </is>
-      </c>
-      <c r="C140" s="1" t="inlineStr">
-        <is>
-          <t>Moonlight glints off the wax.</t>
-        </is>
-      </c>
-      <c r="D140" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E140" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B141" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 5:00 AM and 8:00 AM local time.</t>
-        </is>
-      </c>
-      <c r="C141" s="1" t="inlineStr">
-        <is>
-          <t>The dew hasn't dried and the bees are already at it.</t>
-        </is>
-      </c>
-      <c r="D141" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E141" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B142" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C142" s="1" t="inlineStr">
-        <is>
-          <t>The hive hums with a fresh day's plans.</t>
-        </is>
-      </c>
-      <c r="D142" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E142" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B143" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C143" s="1" t="inlineStr">
-        <is>
-          <t>Even bees pause to enjoy the sunshine.</t>
-        </is>
-      </c>
-      <c r="D143" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E143" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-      <c r="B144" s="1" t="inlineStr">
-        <is>
-          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
-        </is>
-      </c>
-      <c r="C144" s="1" t="inlineStr">
-        <is>
-          <t>Half the day's pollen is already in.</t>
-        </is>
-      </c>
-      <c r="D144" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E144" s="1" t="inlineStr">
-        <is>
-          <t>Loading</t>
         </is>
       </c>
     </row>
@@ -5122,12 +5122,12 @@
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>The hive settles into its afternoon rhythm.</t>
+          <t>Moonlight glints off the wax.</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
@@ -5149,12 +5149,12 @@
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+          <t>Match starts between 5:00 AM and 8:00 AM local time.</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>Long shadows, long odds — let's play.</t>
+          <t>The dew hasn't dried and the bees are already at it.</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
@@ -5176,12 +5176,12 @@
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
+          <t>Match starts between 8:00 AM and 12:00 PM local time.</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>The last foragers are heading home.</t>
+          <t>The hive hums with a fresh day's plans.</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
@@ -5203,12 +5203,12 @@
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
+          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>Lantern-bugs light the way to the hive.</t>
+          <t>Even bees pause to enjoy the sunshine.</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
@@ -5230,12 +5230,12 @@
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 9:00 PM and midnight local time.</t>
+          <t>Match starts between 12:00 PM and 2:00 PM local time.</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>The Queen's chambers go quiet, but not this table.</t>
+          <t>Half the day's pollen is already in.</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
@@ -5257,20 +5257,155 @@
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
+          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C150" s="1" t="inlineStr">
+        <is>
+          <t>The hive settles into its afternoon rhythm.</t>
+        </is>
+      </c>
+      <c r="D150" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E150" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 2:00 PM and 5:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>Long shadows, long odds — let's play.</t>
+        </is>
+      </c>
+      <c r="D151" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E151" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B152" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C152" s="1" t="inlineStr">
+        <is>
+          <t>The last foragers are heading home.</t>
+        </is>
+      </c>
+      <c r="D152" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E152" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B153" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 5:00 PM and 9:00 PM local time.</t>
+        </is>
+      </c>
+      <c r="C153" s="1" t="inlineStr">
+        <is>
+          <t>Lantern-bugs light the way to the hive.</t>
+        </is>
+      </c>
+      <c r="D153" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E153" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B154" s="1" t="inlineStr">
+        <is>
           <t>Match starts between 9:00 PM and midnight local time.</t>
         </is>
       </c>
-      <c r="C150" s="1" t="inlineStr">
+      <c r="C154" s="1" t="inlineStr">
+        <is>
+          <t>The Queen's chambers go quiet, but not this table.</t>
+        </is>
+      </c>
+      <c r="D154" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E154" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B155" s="1" t="inlineStr">
+        <is>
+          <t>Match starts between 9:00 PM and midnight local time.</t>
+        </is>
+      </c>
+      <c r="C155" s="1" t="inlineStr">
         <is>
           <t>A nightcap of nectar before bed.</t>
         </is>
       </c>
-      <c r="D150" s="1" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E150" s="1" t="inlineStr">
+      <c r="D155" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E155" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
         </is>

</xml_diff>

<commit_message>
Add variety to single-message combat/rule banners, normalize punctuation
Adds 2-5 message variants to 24 previously single-message triggers across
Gameplay combat moments and Rule-Specific/Roulette announcements. Normalizes
punctuation to match the catalog's existing conventions along the way:
straight apostrophes, spaced em dashes (not hyphens), unicode ellipses, and
terminal punctuation on every message.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -4251,135 +4251,135 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="inlineStr">
         <is>
           <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="1" t="inlineStr">
         <is>
           <t>A worker bee never doubts their instincts... twice!</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E113" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
         <is>
           <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C114" s="1" t="inlineStr">
         <is>
           <t>Just testing the Undo button, right?</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="inlineStr">
         <is>
           <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="1" t="inlineStr">
         <is>
           <t>You just wanted to see that card flip again!</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
+      <c r="D115" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E115" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
         <is>
           <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="1" t="inlineStr">
         <is>
           <t>A plot twist... that went absolutely nowhere!</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
+      <c r="D116" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E116" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Gameplay</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
         <is>
           <t>Player uses Undo, thinks about it, and then makes the exact same move they just undid.</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="1" t="inlineStr">
         <is>
           <t>Taking the scenic route to the exact same move!</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Repeatable Flavor</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
+      <c r="D117" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E117" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
@@ -5408,6 +5408,1896 @@
       <c r="E155" s="1" t="inlineStr">
         <is>
           <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B156" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C156" s="1" t="inlineStr">
+        <is>
+          <t>Cornered in the comb... can you pull off a miracle?</t>
+        </is>
+      </c>
+      <c r="D156" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E156" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B157" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C157" s="1" t="inlineStr">
+        <is>
+          <t>Down to your final stand! The hive needs a hero.</t>
+        </is>
+      </c>
+      <c r="D157" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E157" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B158" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C158" s="1" t="inlineStr">
+        <is>
+          <t>Only a few cells left! Can a single sting turn the tide?</t>
+        </is>
+      </c>
+      <c r="D158" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E158" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B159" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C159" s="1" t="inlineStr">
+        <is>
+          <t>Trapped in the comb... one last chance to strike back.</t>
+        </is>
+      </c>
+      <c r="D159" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E159" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>Well... this is getting uncomfortable.</t>
+        </is>
+      </c>
+      <c r="D160" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E160" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B161" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C161" s="1" t="inlineStr">
+        <is>
+          <t>Don't panic! ...Okay, maybe panic just a little.</t>
+        </is>
+      </c>
+      <c r="D161" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E161" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B162" s="1" t="inlineStr">
+        <is>
+          <t>Player has only 2 cards on the board vs. opponent's 6, few spaces left.</t>
+        </is>
+      </c>
+      <c r="C162" s="1" t="inlineStr">
+        <is>
+          <t>Backed into a corner — just where we want 'em?</t>
+        </is>
+      </c>
+      <c r="D162" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E162" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B163" s="1" t="inlineStr">
+        <is>
+          <t>Player wins a match with 4 rules active at once.</t>
+        </is>
+      </c>
+      <c r="C163" s="1" t="inlineStr">
+        <is>
+          <t>The odds were quadrupled, and so was your glory!</t>
+        </is>
+      </c>
+      <c r="D163" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E163" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B164" s="1" t="inlineStr">
+        <is>
+          <t>Player wins a match with 4 rules active at once.</t>
+        </is>
+      </c>
+      <c r="C164" s="1" t="inlineStr">
+        <is>
+          <t>Four rules? Just four more reasons to win.</t>
+        </is>
+      </c>
+      <c r="D164" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E164" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B165" s="1" t="inlineStr">
+        <is>
+          <t>Player flips 3+ cards in a single turn.</t>
+        </is>
+      </c>
+      <c r="C165" s="1" t="inlineStr">
+        <is>
+          <t>Sting 'em all!</t>
+        </is>
+      </c>
+      <c r="D165" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E165" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B166" s="1" t="inlineStr">
+        <is>
+          <t>Player flips 3+ cards in a single turn.</t>
+        </is>
+      </c>
+      <c r="C166" s="1" t="inlineStr">
+        <is>
+          <t>Raking in the honey!</t>
+        </is>
+      </c>
+      <c r="D166" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E166" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B167" s="1" t="inlineStr">
+        <is>
+          <t>Player flips 3+ cards in a single turn.</t>
+        </is>
+      </c>
+      <c r="C167" s="1" t="inlineStr">
+        <is>
+          <t>A sweeping sting!</t>
+        </is>
+      </c>
+      <c r="D167" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E167" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B168" s="1" t="inlineStr">
+        <is>
+          <t>Opponent flips 3+ of the player's cards in a single turn (not a Combo).</t>
+        </is>
+      </c>
+      <c r="C168" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} shows no mercy!</t>
+        </is>
+      </c>
+      <c r="D168" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E168" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B169" s="1" t="inlineStr">
+        <is>
+          <t>Opponent flips 3+ of the player's cards in a single turn (not a Combo).</t>
+        </is>
+      </c>
+      <c r="C169" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} didn't hold back!</t>
+        </is>
+      </c>
+      <c r="D169" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E169" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B170" s="1" t="inlineStr">
+        <is>
+          <t>Combo x4 or higher.</t>
+        </is>
+      </c>
+      <c r="C170" s="1" t="inlineStr">
+        <is>
+          <t>MEGA CASCADE — absolute hive pandemonium!</t>
+        </is>
+      </c>
+      <c r="D170" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E170" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B171" s="1" t="inlineStr">
+        <is>
+          <t>Combo x4 or higher.</t>
+        </is>
+      </c>
+      <c r="C171" s="1" t="inlineStr">
+        <is>
+          <t>HIVE SUPERNOVA — a four-fold combo explosion!</t>
+        </is>
+      </c>
+      <c r="D171" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E171" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B172" s="1" t="inlineStr">
+        <is>
+          <t>Combo x4 or higher.</t>
+        </is>
+      </c>
+      <c r="C172" s="1" t="inlineStr">
+        <is>
+          <t>ULTIMATE SWARM — cards flipping in every direction!</t>
+        </is>
+      </c>
+      <c r="D172" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E172" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B173" s="1" t="inlineStr">
+        <is>
+          <t>A placed card captures on all 4 sides at once.</t>
+        </is>
+      </c>
+      <c r="C173" s="1" t="inlineStr">
+        <is>
+          <t>Omnidirectional sting — nothing on that board was safe!</t>
+        </is>
+      </c>
+      <c r="D173" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E173" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B174" s="1" t="inlineStr">
+        <is>
+          <t>A placed card captures on all 4 sides at once.</t>
+        </is>
+      </c>
+      <c r="C174" s="1" t="inlineStr">
+        <is>
+          <t>Royal center sting!</t>
+        </is>
+      </c>
+      <c r="D174" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E174" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B175" s="1" t="inlineStr">
+        <is>
+          <t>A placed card captures on all 4 sides at once.</t>
+        </is>
+      </c>
+      <c r="C175" s="1" t="inlineStr">
+        <is>
+          <t>Bullseye in the comb!</t>
+        </is>
+      </c>
+      <c r="D175" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E175" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B176" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C176" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName}'s wings are getting tired!</t>
+        </is>
+      </c>
+      <c r="D176" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E176" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B177" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C177" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} is losing their buzz!</t>
+        </is>
+      </c>
+      <c r="D177" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E177" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B178" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C178" s="1" t="inlineStr">
+        <is>
+          <t>You're ruling this hive!</t>
+        </is>
+      </c>
+      <c r="D178" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E178" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B179" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C179" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} can't catch a break.</t>
+        </is>
+      </c>
+      <c r="D179" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E179" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B180" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch wins in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C180" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} might need a quick coffee break.</t>
+        </is>
+      </c>
+      <c r="D180" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E180" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B181" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch losses in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C181" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} is on a roll… time to shake up your deck!</t>
+        </is>
+      </c>
+      <c r="D181" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E181" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B182" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch losses in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C182" s="1" t="inlineStr">
+        <is>
+          <t>Smoked out by {OpponentName} 3 times in a row!</t>
+        </is>
+      </c>
+      <c r="D182" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E182" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B183" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch losses in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C183" s="1" t="inlineStr">
+        <is>
+          <t>The swarm is favoring {OpponentName}… for now!</t>
+        </is>
+      </c>
+      <c r="D183" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E183" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B184" s="1" t="inlineStr">
+        <is>
+          <t>3+ rematch losses in a row against the same opponent.</t>
+        </is>
+      </c>
+      <c r="C184" s="1" t="inlineStr">
+        <is>
+          <t>Got caught in {OpponentName}'s honey trap again!</t>
+        </is>
+      </c>
+      <c r="D184" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E184" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B185" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures 3+ cards in one move.</t>
+        </is>
+      </c>
+      <c r="C185" s="1" t="inlineStr">
+        <is>
+          <t>A humble worker bee just staged a revolution!</t>
+        </is>
+      </c>
+      <c r="D185" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E185" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B186" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures 3+ cards in one move.</t>
+        </is>
+      </c>
+      <c r="C186" s="1" t="inlineStr">
+        <is>
+          <t>Smallest bee, ENORMOUS sting!</t>
+        </is>
+      </c>
+      <c r="D186" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E186" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B187" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures 3+ cards in one move.</t>
+        </is>
+      </c>
+      <c r="C187" s="1" t="inlineStr">
+        <is>
+          <t>Don't judge a bee by its stars!</t>
+        </is>
+      </c>
+      <c r="D187" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E187" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B188" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures 3+ cards in one move.</t>
+        </is>
+      </c>
+      <c r="C188" s="1" t="inlineStr">
+        <is>
+          <t>Small card, big moves!</t>
+        </is>
+      </c>
+      <c r="D188" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E188" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B189" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
+        </is>
+      </c>
+      <c r="C189" s="1" t="inlineStr">
+        <is>
+          <t>The ultimate rarity mismatch!</t>
+        </is>
+      </c>
+      <c r="D189" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E189" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B190" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
+        </is>
+      </c>
+      <c r="C190" s="1" t="inlineStr">
+        <is>
+          <t>Rank means nothing to a sharp stinger!</t>
+        </is>
+      </c>
+      <c r="D190" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E190" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B191" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
+        </is>
+      </c>
+      <c r="C191" s="1" t="inlineStr">
+        <is>
+          <t>Royalty is expensive — tactics are free!</t>
+        </is>
+      </c>
+      <c r="D191" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E191" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B192" s="1" t="inlineStr">
+        <is>
+          <t>A 1-star card captures a 5-star card (rarity mismatch).</t>
+        </is>
+      </c>
+      <c r="C192" s="1" t="inlineStr">
+        <is>
+          <t>Big stars fall hard!</t>
+        </is>
+      </c>
+      <c r="D192" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E192" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B193" s="1" t="inlineStr">
+        <is>
+          <t>Player plays against the same AI difficulty 5 times in a row.</t>
+        </is>
+      </c>
+      <c r="C193" s="1" t="inlineStr">
+        <is>
+          <t>Neither bee backs down — 5 matches and counting!</t>
+        </is>
+      </c>
+      <c r="D193" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E193" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B194" s="1" t="inlineStr">
+        <is>
+          <t>Player plays against the same AI difficulty 5 times in a row.</t>
+        </is>
+      </c>
+      <c r="C194" s="1" t="inlineStr">
+        <is>
+          <t>Five battles in the same comb! The bees are watching closely.</t>
+        </is>
+      </c>
+      <c r="D194" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E194" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B195" s="1" t="inlineStr">
+        <is>
+          <t>Player plays against the same AI difficulty 5 times in a row.</t>
+        </is>
+      </c>
+      <c r="C195" s="1" t="inlineStr">
+        <is>
+          <t>Deep in the hive, a classic matchup unfolds.</t>
+        </is>
+      </c>
+      <c r="D195" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E195" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B196" s="1" t="inlineStr">
+        <is>
+          <t>Player wins by the maximum possible margin.</t>
+        </is>
+      </c>
+      <c r="C196" s="1" t="inlineStr">
+        <is>
+          <t>Absolute hive takeover!</t>
+        </is>
+      </c>
+      <c r="D196" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E196" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B197" s="1" t="inlineStr">
+        <is>
+          <t>Player wins by the maximum possible margin.</t>
+        </is>
+      </c>
+      <c r="C197" s="1" t="inlineStr">
+        <is>
+          <t>All the honey is yours!</t>
+        </is>
+      </c>
+      <c r="D197" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E197" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="B198" s="1" t="inlineStr">
+        <is>
+          <t>Player wins by the maximum possible margin.</t>
+        </is>
+      </c>
+      <c r="C198" s="1" t="inlineStr">
+        <is>
+          <t>Not even a drone left standing!</t>
+        </is>
+      </c>
+      <c r="D198" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E198" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B199" s="1" t="inlineStr">
+        <is>
+          <t>Nectar Exchange swaps away the player's 5-star card.</t>
+        </is>
+      </c>
+      <c r="C199" s="1" t="inlineStr">
+        <is>
+          <t>{OpponentName} just flew off with your Royal Jelly!</t>
+        </is>
+      </c>
+      <c r="D199" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E199" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B200" s="1" t="inlineStr">
+        <is>
+          <t>Nectar Exchange swaps away the player's 5-star card.</t>
+        </is>
+      </c>
+      <c r="C200" s="1" t="inlineStr">
+        <is>
+          <t>Highway robbery in the hive! {OpponentName} stole your 5-star!</t>
+        </is>
+      </c>
+      <c r="D200" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E200" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B201" s="1" t="inlineStr">
+        <is>
+          <t>Nectar Exchange trades the player's worst card for the opponent's best.</t>
+        </is>
+      </c>
+      <c r="C201" s="1" t="inlineStr">
+        <is>
+          <t>The nectar favors you.</t>
+        </is>
+      </c>
+      <c r="D201" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E201" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B202" s="1" t="inlineStr">
+        <is>
+          <t>Nectar Exchange trades the player's worst card for the opponent's best.</t>
+        </is>
+      </c>
+      <c r="C202" s="1" t="inlineStr">
+        <is>
+          <t>A golden exchange.</t>
+        </is>
+      </c>
+      <c r="D202" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E202" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B203" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls zero extra rules.</t>
+        </is>
+      </c>
+      <c r="C203" s="1" t="inlineStr">
+        <is>
+          <t>Pure, unadulterated honey — standard rules apply!</t>
+        </is>
+      </c>
+      <c r="D203" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E203" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B204" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls zero extra rules.</t>
+        </is>
+      </c>
+      <c r="C204" s="1" t="inlineStr">
+        <is>
+          <t>Back to basics for the bees!</t>
+        </is>
+      </c>
+      <c r="D204" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E204" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B205" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls zero extra rules.</t>
+        </is>
+      </c>
+      <c r="C205" s="1" t="inlineStr">
+        <is>
+          <t>Clean comb, clean rules — just you and the cards.</t>
+        </is>
+      </c>
+      <c r="D205" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E205" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B206" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Pollination.</t>
+        </is>
+      </c>
+      <c r="C206" s="1" t="inlineStr">
+        <is>
+          <t>Flowers are blooming!</t>
+        </is>
+      </c>
+      <c r="D206" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E206" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B207" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Pollination.</t>
+        </is>
+      </c>
+      <c r="C207" s="1" t="inlineStr">
+        <is>
+          <t>Pollen. Everywhere.</t>
+        </is>
+      </c>
+      <c r="D207" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E207" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B208" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Smoked Out.</t>
+        </is>
+      </c>
+      <c r="C208" s="1" t="inlineStr">
+        <is>
+          <t>Smoke fills the hive…</t>
+        </is>
+      </c>
+      <c r="D208" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E208" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B209" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Math Bee</t>
+        </is>
+      </c>
+      <c r="C209" s="1" t="inlineStr">
+        <is>
+          <t>Do the math!</t>
+        </is>
+      </c>
+      <c r="D209" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E209" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B210" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Math Bee</t>
+        </is>
+      </c>
+      <c r="C210" s="1" t="inlineStr">
+        <is>
+          <t>Sum it up!</t>
+        </is>
+      </c>
+      <c r="D210" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E210" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B211" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Math Bee</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="inlineStr">
+        <is>
+          <t>Calculate carefully!</t>
+        </is>
+      </c>
+      <c r="D211" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E211" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B212" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Math Bee</t>
+        </is>
+      </c>
+      <c r="C212" s="1" t="inlineStr">
+        <is>
+          <t>Class is in session!</t>
+        </is>
+      </c>
+      <c r="D212" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E212" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B213" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Inversion</t>
+        </is>
+      </c>
+      <c r="C213" s="1" t="inlineStr">
+        <is>
+          <t>Flying backwards — low beats high!</t>
+        </is>
+      </c>
+      <c r="D213" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E213" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B214" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls clear skies</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="inlineStr">
+        <is>
+          <t>Clear Skies overheard.</t>
+        </is>
+      </c>
+      <c r="D214" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E214" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B215" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls clear skies</t>
+        </is>
+      </c>
+      <c r="C215" s="1" t="inlineStr">
+        <is>
+          <t>No shade on the hive today.</t>
+        </is>
+      </c>
+      <c r="D215" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E215" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B216" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls scouting party</t>
+        </is>
+      </c>
+      <c r="C216" s="1" t="inlineStr">
+        <is>
+          <t>Scout bees have reported back!</t>
+        </is>
+      </c>
+      <c r="D216" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E216" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B217" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls scouting party</t>
+        </is>
+      </c>
+      <c r="C217" s="1" t="inlineStr">
+        <is>
+          <t>Reconnaissance in progress!</t>
+        </is>
+      </c>
+      <c r="D217" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E217" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B218" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls scouting party</t>
+        </is>
+      </c>
+      <c r="C218" s="1" t="inlineStr">
+        <is>
+          <t>Intel gathered!</t>
+        </is>
+      </c>
+      <c r="D218" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E218" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B219" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Frenzy</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="inlineStr">
+        <is>
+          <t>The bees are out of control!</t>
+        </is>
+      </c>
+      <c r="D219" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E219" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B220" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Frenzy</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="inlineStr">
+        <is>
+          <t>Those bees are wild!</t>
+        </is>
+      </c>
+      <c r="D220" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E220" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B221" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Symmetry</t>
+        </is>
+      </c>
+      <c r="C221" s="1" t="inlineStr">
+        <is>
+          <t>Geometric precision required.</t>
+        </is>
+      </c>
+      <c r="D221" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E221" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B222" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Nectar Exchange</t>
+        </is>
+      </c>
+      <c r="C222" s="1" t="inlineStr">
+        <is>
+          <t>Pre-game trading post open!</t>
+        </is>
+      </c>
+      <c r="D222" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E222" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B223" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Nectar Exchange</t>
+        </is>
+      </c>
+      <c r="C223" s="1" t="inlineStr">
+        <is>
+          <t>Nectar bartering begins!</t>
+        </is>
+      </c>
+      <c r="D223" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E223" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B224" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Hierarchy</t>
+        </is>
+      </c>
+      <c r="C224" s="1" t="inlineStr">
+        <is>
+          <t>Obey the Queen!</t>
+        </is>
+      </c>
+      <c r="D224" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E224" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B225" s="1" t="inlineStr">
+        <is>
+          <t>Roulette rolls Hierarchy</t>
+        </is>
+      </c>
+      <c r="C225" s="1" t="inlineStr">
+        <is>
+          <t>Royal decree issued!</t>
+        </is>
+      </c>
+      <c r="D225" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E225" s="1" t="inlineStr">
+        <is>
+          <t>Game intro rules banner</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close loading-banner time gap, fix Windows event-subscription leak
- Extend the Late Night loading-banner window from 12:00-4:00am to
  12:00-5:00am on both platforms, closing a silent gap where a 4am app
  launch fell through to the generic fallback instead of a time-specific
  banner.
- Fix HoneycombView (Windows) never unsubscribing from its ViewModel's
  events on Unloaded, unlike every sibling game view. Since MainWindow
  caches and reattaches this view on every game switch, Loaded fires on
  each reattach — without Unloaded, repeated switching back to Honeycomb
  stacked duplicate subscriptions, causing banners/refreshes/swap effects
  to fire multiple times per real event.
- Clean up two stale/misplaced comments left behind by earlier refactors
  in HoneycombViewModel.cs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>Match starts between 12:00 AM and 4:00 AM local time.</t>
+          <t>Match starts between 12:00 AM and 5:00 AM local time.</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add Valentine's suit toasts, more April Fools lines, and 10 new holidays
Content additions to the Loading/Valentine's Day trigger (11 new suit-themed
messages) and April Fools trigger (4 new lines), plus 10 new named
holidays: Earth Day, National Honey Day, Pi Day, New Year's Eve, Christmas
(fixed Gregorian dates), and Holi, Rosh Hashanah, Diwali, Eid al-Fitr,
Hanukkah (lunisolar/lunar — added via a 20-year per-year date lookup table,
2025-2045, inline in the existing loadingBannerID()/LoadingBannerId()
holiday ladder rather than a new service, matching how every other holiday
in the catalog already works). Each floating holiday's table lists only its
first day, since multi-day observances should only trigger the banner once.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E225"/>
+  <dimension ref="A1:E250"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -7298,6 +7298,681 @@
       <c r="E225" s="1" t="inlineStr">
         <is>
           <t>Game intro rules banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B226" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C226" s="1" t="inlineStr">
+        <is>
+          <t>Hearts flutter through the hive today.</t>
+        </is>
+      </c>
+      <c r="D226" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E226" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B227" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C227" s="1" t="inlineStr">
+        <is>
+          <t>Every heart in the comb beats a little louder.</t>
+        </is>
+      </c>
+      <c r="D227" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E227" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B228" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C228" s="1" t="inlineStr">
+        <is>
+          <t>The hive is full of hearts, and yours is winning.</t>
+        </is>
+      </c>
+      <c r="D228" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E228" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B229" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C229" s="1" t="inlineStr">
+        <is>
+          <t>Diamonds sparkle brighter on Valentine's Day.</t>
+        </is>
+      </c>
+      <c r="D229" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E229" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B230" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="inlineStr">
+        <is>
+          <t>The bees traded honey for diamonds today.</t>
+        </is>
+      </c>
+      <c r="D230" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E230" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B231" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C231" s="1" t="inlineStr">
+        <is>
+          <t>A diamond in the rough, sweeter than honey.</t>
+        </is>
+      </c>
+      <c r="D231" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E231" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B232" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C232" s="1" t="inlineStr">
+        <is>
+          <t>Clover and clubs bloom together this Valentine's.</t>
+        </is>
+      </c>
+      <c r="D232" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E232" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B233" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C233" s="1" t="inlineStr">
+        <is>
+          <t>Even the clubs are feeling the love today.</t>
+        </is>
+      </c>
+      <c r="D233" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E233" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B234" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C234" s="1" t="inlineStr">
+        <is>
+          <t>Cupid's arrow struck the spades first.</t>
+        </is>
+      </c>
+      <c r="D234" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E234" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B235" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C235" s="1" t="inlineStr">
+        <is>
+          <t>The spades soften their edges for Valentine's Day.</t>
+        </is>
+      </c>
+      <c r="D235" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E235" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B236" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Valentine's Day (Feb 14).</t>
+        </is>
+      </c>
+      <c r="C236" s="1" t="inlineStr">
+        <is>
+          <t>Even spades dig deep for love today.</t>
+        </is>
+      </c>
+      <c r="D236" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E236" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B237" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Earth Day (Apr 22).</t>
+        </is>
+      </c>
+      <c r="C237" s="1" t="inlineStr">
+        <is>
+          <t>Protect the flowers, save the bees! Happy Earth Day!</t>
+        </is>
+      </c>
+      <c r="D237" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E237" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B238" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on National Honey Day (Aug 15).</t>
+        </is>
+      </c>
+      <c r="C238" s="1" t="inlineStr">
+        <is>
+          <t>A golden celebration in the comb — Happy Honey Day!</t>
+        </is>
+      </c>
+      <c r="D238" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E238" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B239" s="1" t="inlineStr">
+        <is>
+          <t>Playing on April Fools' Day (Apr 1).</t>
+        </is>
+      </c>
+      <c r="C239" s="1" t="inlineStr">
+        <is>
+          <t>Is that card really what it seems… or an April Fools' trick?</t>
+        </is>
+      </c>
+      <c r="D239" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E239" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B240" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Pi Day (Mar 14).</t>
+        </is>
+      </c>
+      <c r="C240" s="1" t="inlineStr">
+        <is>
+          <t>The math in the comb is extra precise today!</t>
+        </is>
+      </c>
+      <c r="D240" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E240" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B241" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on New Year's Eve (Dec 31).</t>
+        </is>
+      </c>
+      <c r="C241" s="1" t="inlineStr">
+        <is>
+          <t>Counting down the final buzz of the year!</t>
+        </is>
+      </c>
+      <c r="D241" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E241" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B242" s="1" t="inlineStr">
+        <is>
+          <t>Game loads on Christmas (Dec 25).</t>
+        </is>
+      </c>
+      <c r="C242" s="1" t="inlineStr">
+        <is>
+          <t>Peace, warmth, and sweetness to all in the hive this Christmas!</t>
+        </is>
+      </c>
+      <c r="D242" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E242" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B243" s="1" t="inlineStr">
+        <is>
+          <t>Playing on April Fools' Day (Apr 1).</t>
+        </is>
+      </c>
+      <c r="C243" s="1" t="inlineStr">
+        <is>
+          <t>Is that a 5-star card, or just a worker bee in a fake crown?</t>
+        </is>
+      </c>
+      <c r="D243" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E243" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B244" s="1" t="inlineStr">
+        <is>
+          <t>Playing on April Fools' Day (Apr 1).</t>
+        </is>
+      </c>
+      <c r="C244" s="1" t="inlineStr">
+        <is>
+          <t>Maybe it's time for a wasp theme…</t>
+        </is>
+      </c>
+      <c r="D244" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E244" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B245" s="1" t="inlineStr">
+        <is>
+          <t>Playing on April Fools' Day (Apr 1).</t>
+        </is>
+      </c>
+      <c r="C245" s="1" t="inlineStr">
+        <is>
+          <t>Pranksters in the hive! Trust your cards, not the drones.</t>
+        </is>
+      </c>
+      <c r="D245" s="1" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E245" s="1" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Game loads on Holi.</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Vibrant colors bloom across the comb! Happy Holi!</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Game loads on Rosh Hashanah.</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Wishing you a sweet and fruitful new year — Shanah Tovah from the hive!</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Game loads on Diwali.</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Wishing you a season of light, sweetness, and harmony in the hive.</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Game loads on Eid al-Fitr.</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>A season of gratitude, sweetness, and joy. Eid Mubarak from the hive!</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Game loads on Hanukkah.</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>May your home bee filled with light, peace, and joy this Hanukkah.</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Loading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update two milestone banners and add variants for three repeatable-flavor banners
Welcome/1000-wins milestone text refreshed; Plus combo, Pollination, and
Smoked Out each gain additional rotating message variants. Edited via
tools/Honeycomb_Fun_Messages.xlsx and regenerated both platforms' catalog
JSON with tools/generate_banner_catalog.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E258"/>
+  <dimension ref="A1:E262"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>A new bee joins the hive. Thank you for playing!</t>
+          <t>Welcome to the colony! Time to make some honey.</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>1000 wins. The hive bends to your will.</t>
+          <t>1000 wins. A millennium of triumph. The Queen herself applauds.</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
@@ -8004,189 +8004,297 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" t="inlineStr">
+      <c r="A252" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr">
+      <c r="B252" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C252" t="inlineStr">
+      <c r="C252" s="1" t="inlineStr">
         <is>
           <t>Calculating 475 moves ahead, or taking a snack break?</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr">
+      <c r="D252" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr">
+      <c r="E252" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" t="inlineStr">
+      <c r="A253" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
+      <c r="B253" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr">
+      <c r="C253" s="1" t="inlineStr">
         <is>
           <t>The cards aren't going to play themselves… though that would be a neat.</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr">
+      <c r="D253" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr">
+      <c r="E253" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="254">
-      <c r="A254" t="inlineStr">
+      <c r="A254" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr">
+      <c r="B254" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr">
+      <c r="C254" s="1" t="inlineStr">
         <is>
           <t>Checking your hand twice? Santa Bee would be proud.</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr">
+      <c r="D254" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
+      <c r="E254" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="255">
-      <c r="A255" t="inlineStr">
+      <c r="A255" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr">
+      <c r="B255" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr">
+      <c r="C255" s="1" t="inlineStr">
         <is>
           <t>No pressure, it's only the entire match on the line.</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr">
+      <c r="D255" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr">
+      <c r="E255" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="256">
-      <c r="A256" t="inlineStr">
+      <c r="A256" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
+      <c r="B256" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr">
+      <c r="C256" s="1" t="inlineStr">
         <is>
           <t>A masterclass in the dramatic pause.</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr">
+      <c r="D256" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr">
+      <c r="E256" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="257">
-      <c r="A257" t="inlineStr">
+      <c r="A257" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
+      <c r="B257" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr">
+      <c r="C257" s="1" t="inlineStr">
         <is>
           <t>Shuffling your thoughts? We've got time.</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr">
+      <c r="D257" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr">
+      <c r="E257" s="1" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>
       </c>
     </row>
     <row r="258">
-      <c r="A258" t="inlineStr">
+      <c r="A258" s="1" t="inlineStr">
         <is>
           <t>Idle Action</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr">
+      <c r="B258" s="1" t="inlineStr">
         <is>
           <t>No action taken for one minute.</t>
         </is>
       </c>
-      <c r="C258" t="inlineStr">
+      <c r="C258" s="1" t="inlineStr">
         <is>
           <t>Brain.exe is processing the optimal placement…</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr">
+      <c r="D258" s="1" t="inlineStr">
         <is>
           <t>Ambiance</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr">
+      <c r="E258" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>A player triggers a "Plus" combo (the math matches perfectly).</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Calculated to perfection!</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Pollination pushes a card's modifier to +3 or higher.</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>{AscensionSuit} is drowning in nectar!</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Pollination pushes a card's modifier to +3 or higher.</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>A massive harvest! {AscensionSuit} thrives.</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Rule-Specific</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Smoked Out drops a card's effective stat to 1.</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Lethargic and grounded.</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Repeatable Flavor</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>

</xml_diff>

<commit_message>
Add 26 new idle-toast messages (clickbait headlines + bee-pun quotes/idioms)
Appended to the existing "no action taken for one minute" catalog entry
alongside the current idle ambiance messages.
</commit_message>
<xml_diff>
--- a/tools/Honeycomb_Fun_Messages.xlsx
+++ b/tools/Honeycomb_Fun_Messages.xlsx
@@ -1216,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E262"/>
+  <dimension ref="A1:E288"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="21.3516" customWidth="1" style="1" min="1" max="1"/>
@@ -8295,6 +8295,708 @@
         </is>
       </c>
       <c r="E262" s="1" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Has science gone too far? Click here to see this 10-star card.</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Local worker bee discovers secret to endless nectar...</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Top 10 cards to steal from the Queen. Number 4 will sting you!</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Beekeepers will hate you! Win every match with this one simple trick!</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Get rich or buzz trying.</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>To bee, or not to bee... wait, whose turn is it?</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>May the swarm be with you.</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Live, Laugh, Pollinate.</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Keep calm and buzz on.</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Home is where the hive is.</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Just a worker bee looking for my queen.</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Are you gonna play a card, or just sit there looking sweet?</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Frankly, my dear, I don't give a buzz.</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>We're gonna need a bigger hive.</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Show me the honey!</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>I'll bee back.</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Nobody puts Baby Bee in a corner.</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Sweet dreams are made of bees.</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Bee yourself; everyone else is already taken.</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Mind your own beeswax!</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>This one weird trick captures 4 cards at once — dealers don't want you to know it.</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>You won't believe what happened when a worker bee met a Fallen Ace.</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>She said yes to Symmetry. He said yes to Math Bee. Chaos ensued.</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Busy as a bee, broke as a beekeeper.</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Absence makes the heart grow fonder — and the hive grow louder.</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Idle Action</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>No action taken for one minute.</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Two bees or not two bees — that's a math problem, not a question.</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Ambiance</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
         <is>
           <t>Toast</t>
         </is>

</xml_diff>